<commit_message>
Put Unit next to units/packet in the Excel template and rename stock to opening stock at 0.
All kitchen-chart items stay in the file. pc/g sit under the Unit column, not under the price columns.

Co-authored-by: vigni2104 <vigni2104@gmail.com>
</commit_message>
<xml_diff>
--- a/assets/templates/menu_items_import.xlsx
+++ b/assets/templates/menu_items_import.xlsx
@@ -71,12 +71,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -448,16 +451,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,22 +501,22 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>stock</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>opening stock</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>cost_price</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>selling_price</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>unit</t>
         </is>
       </c>
     </row>
@@ -545,13 +548,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -581,13 +587,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -617,13 +626,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -653,13 +665,16 @@
           <t>50</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -689,13 +704,16 @@
           <t>50</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -725,13 +743,16 @@
           <t>28</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -761,13 +782,16 @@
           <t>8</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -797,13 +821,16 @@
           <t>13</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -833,13 +860,16 @@
           <t>40</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -869,13 +899,16 @@
           <t>20</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -905,13 +938,16 @@
           <t>39</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -941,13 +977,16 @@
           <t>60</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -977,13 +1016,16 @@
           <t>27</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1013,13 +1055,16 @@
           <t>50</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1049,13 +1094,16 @@
           <t>33</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1085,13 +1133,16 @@
           <t>28</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1121,13 +1172,16 @@
           <t>14</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1157,13 +1211,16 @@
           <t>2500</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>g</t>
         </is>
       </c>
+      <c r="I19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1193,13 +1250,16 @@
           <t>13</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1229,13 +1289,16 @@
           <t>13</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1265,13 +1328,16 @@
           <t>5</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1301,13 +1367,16 @@
           <t>6</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1337,13 +1406,16 @@
           <t>6</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1369,12 +1441,16 @@
       </c>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1400,12 +1476,16 @@
       </c>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1431,12 +1511,16 @@
       </c>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1462,12 +1546,16 @@
       </c>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1493,12 +1581,16 @@
       </c>
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1524,12 +1616,16 @@
       </c>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1555,12 +1651,16 @@
       </c>
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K31"/>

</xml_diff>

<commit_message>
Encode Chicken Popcorn as 69 g per sale and 552 g per packet.
Matches the chart: 8 portions per pack times 69 g per portion.

Co-authored-by: vigni2104 <vigni2104@gmail.com>
</commit_message>
<xml_diff>
--- a/assets/templates/menu_items_import.xlsx
+++ b/assets/templates/menu_items_import.xlsx
@@ -773,18 +773,18 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>69</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>552</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>pc</t>
+          <t>g</t>
         </is>
       </c>
       <c r="I8" s="3" t="n">

</xml_diff>

<commit_message>
Load all 30 kitchen-chart items from the converted menu file.
Seed from CSV so every row is added, rebuild the Excel with the same list, and keep Chicken Popcorn as 69 g per sale.

Co-authored-by: vigni2104 <vigni2104@gmail.com>
</commit_message>
<xml_diff>
--- a/assets/templates/menu_items_import.xlsx
+++ b/assets/templates/menu_items_import.xlsx
@@ -536,17 +536,13 @@
           <t>Thai Crispy</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -556,8 +552,8 @@
       <c r="I2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -575,17 +571,13 @@
           <t>Crunchy Masala</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -595,8 +587,8 @@
       <c r="I3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -614,17 +606,13 @@
           <t>Chilli Burst</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -634,8 +622,8 @@
       <c r="I4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -653,17 +641,13 @@
           <t>Krusty Bites</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n">
+        <v>50</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -673,8 +657,8 @@
       <c r="I5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -692,17 +676,13 @@
           <t>Chicken 65</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n">
+        <v>50</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -712,8 +692,8 @@
       <c r="I6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -731,17 +711,13 @@
           <t>Peri Peri Chwings</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n">
+        <v>28</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -751,8 +727,8 @@
       <c r="I7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -770,17 +746,13 @@
           <t>Chicken Popcorn</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>552</t>
-        </is>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n">
+        <v>552</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -790,8 +762,8 @@
       <c r="I8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -809,17 +781,13 @@
           <t>Whole Muscle Patty</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n">
+        <v>13</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -829,8 +797,8 @@
       <c r="I9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -848,17 +816,13 @@
           <t>Chicken Momos</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n">
+        <v>40</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -868,8 +832,8 @@
       <c r="I10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -887,17 +851,13 @@
           <t>Crispy Chicken Patty</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n">
+        <v>20</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -907,8 +867,8 @@
       <c r="I11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -926,17 +886,13 @@
           <t>Chicken Fingers</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n">
+        <v>39</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -946,8 +902,8 @@
       <c r="I12" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -965,17 +921,13 @@
           <t>Chicken Nuggets</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n">
+        <v>60</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -985,8 +937,8 @@
       <c r="I13" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1004,17 +956,13 @@
           <t>Chicken Strips</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n">
+        <v>27</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1024,8 +972,8 @@
       <c r="I14" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1043,17 +991,13 @@
           <t>Chicken Cheese Shotz</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n">
+        <v>50</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1063,8 +1007,8 @@
       <c r="I15" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1082,17 +1026,13 @@
           <t>Veg Finger</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n">
+        <v>33</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1102,8 +1042,8 @@
       <c r="I16" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1121,17 +1061,13 @@
           <t>Pizza Pocket</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n">
+        <v>28</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1141,8 +1077,8 @@
       <c r="I17" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1160,17 +1096,13 @@
           <t>Paneer Patty</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n">
+        <v>14</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1180,8 +1112,8 @@
       <c r="I18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1199,17 +1131,13 @@
           <t>French Fries</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>2500</t>
-        </is>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n">
+        <v>2500</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1219,8 +1147,8 @@
       <c r="I19" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1238,17 +1166,13 @@
           <t>Veg Patty</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n">
+        <v>13</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1258,8 +1182,8 @@
       <c r="I20" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1277,17 +1201,13 @@
           <t>Tandoori Patty</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n">
+        <v>13</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1297,8 +1217,8 @@
       <c r="I21" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1316,17 +1236,13 @@
           <t>Hot Crispy Patty</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1336,8 +1252,8 @@
       <c r="I22" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1355,17 +1271,13 @@
           <t>Burger Bun With Sesame</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1375,8 +1287,8 @@
       <c r="I23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1394,17 +1306,13 @@
           <t>Plain Burger Bun</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1414,8 +1322,8 @@
       <c r="I24" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1433,14 +1341,12 @@
           <t>Tandoori Filling</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1449,8 +1355,8 @@
       <c r="I25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1468,14 +1374,12 @@
           <t>Paratha</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1484,8 +1388,8 @@
       <c r="I26" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1503,14 +1407,12 @@
           <t>Paratha Sauce</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1519,8 +1421,8 @@
       <c r="I27" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1538,14 +1440,12 @@
           <t>Eggless Mayonnaise</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1554,8 +1454,8 @@
       <c r="I28" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1573,14 +1473,12 @@
           <t>Tandoori Mayonnaise</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1589,8 +1487,8 @@
       <c r="I29" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1608,14 +1506,12 @@
           <t>BBQ Seasoning</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1624,8 +1520,8 @@
       <c r="I30" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1643,14 +1539,12 @@
           <t>CP Marinade</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr"/>
-      <c r="G31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1659,8 +1553,8 @@
       <c r="I31" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K31"/>

</xml_diff>